<commit_message>
Filter collaborators by active status
</commit_message>
<xml_diff>
--- a/Base de colaboradores.xlsx
+++ b/Base de colaboradores.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\SERVER_ANTIGO\SETOR DE COBRANÇA\BASE DE DADOS\NEGOCIADORES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samuel.victor\Desktop\ANALISE DO HISTORICO DE OPERADORES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C2F8966-6E2D-4ECF-9814-4C4D5A75699A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A76E6B45-DF0F-468A-A355-49A330A08F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-2490" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-3270" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="JUDICIAL" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,9 @@
     <sheet name="ITAPEVA" sheetId="2" r:id="rId3"/>
     <sheet name="ADM" sheetId="3" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">JUDICIAL!$A$18:$I$32</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -37,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="182">
   <si>
     <t>NOME COLABORADOR</t>
   </si>
@@ -574,6 +577,15 @@
   </si>
   <si>
     <t>brenner.merencio</t>
+  </si>
+  <si>
+    <t>ATIVO</t>
+  </si>
+  <si>
+    <t>NÃO</t>
+  </si>
+  <si>
+    <t>SIM</t>
   </si>
 </sst>
 </file>
@@ -613,15 +625,21 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -740,6 +758,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -752,7 +785,7 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -829,6 +862,15 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -841,7 +883,52 @@
     <cellStyle name="Vírgula 2" xfId="5" xr:uid="{9CDD5147-56E3-4C33-9F03-D920CCE161A2}"/>
     <cellStyle name="Vírgula 3" xfId="8" xr:uid="{2B217E81-60B0-4E52-ABFD-A7D055F17E6E}"/>
   </cellStyles>
-  <dxfs count="54">
+  <dxfs count="55">
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -871,6 +958,216 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
@@ -1454,238 +1751,6 @@
       <border outline="0">
         <bottom style="thin">
           <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
         </bottom>
       </border>
     </dxf>
@@ -1716,67 +1781,68 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E73478C6-AA34-456B-BB72-ADF60DB89795}" name="Tabela2" displayName="Tabela2" ref="A1:H17" totalsRowShown="0" headerRowDxfId="53" dataDxfId="51" headerRowBorderDxfId="52" tableBorderDxfId="50" totalsRowBorderDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E73478C6-AA34-456B-BB72-ADF60DB89795}" name="Tabela2" displayName="Tabela2" ref="A1:I17" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" headerRowBorderDxfId="13" tableBorderDxfId="14" totalsRowBorderDxfId="12">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H16">
     <sortCondition ref="A15:A16"/>
   </sortState>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{44B01074-0E94-49D7-A638-9DE941BE9A75}" name="NOME COLABORADOR" dataDxfId="48"/>
-    <tableColumn id="5" xr3:uid="{F9A57807-E92F-4AC4-A57B-5E3A31CA8C2B}" name="LOGIN COBMAIS" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{3D537BF0-580E-42DC-AAC3-452BD19ECF16}" name="ID SRS" dataDxfId="46"/>
-    <tableColumn id="6" xr3:uid="{AE32C28F-E44F-4C85-B0D8-0877E06AAD05}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="45" dataCellStyle="Hiperlink"/>
-    <tableColumn id="3" xr3:uid="{62104941-F9E6-4824-97B5-2A48ACFEB884}" name="DATA ADMISSÃO" dataDxfId="44"/>
-    <tableColumn id="8" xr3:uid="{7271809A-319F-42CA-B3C0-541D631C23AA}" name="CARGO" dataDxfId="43"/>
-    <tableColumn id="7" xr3:uid="{0D375E2B-128D-4616-9AC4-B297337904BE}" name="GÊNERO" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{D8BE0E60-84AD-463D-A75B-55784F722626}" name="DATA DE NASCIMENTO" dataDxfId="41"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{44B01074-0E94-49D7-A638-9DE941BE9A75}" name="NOME COLABORADOR" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{F9A57807-E92F-4AC4-A57B-5E3A31CA8C2B}" name="LOGIN COBMAIS" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{3D537BF0-580E-42DC-AAC3-452BD19ECF16}" name="ID SRS" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{AE32C28F-E44F-4C85-B0D8-0877E06AAD05}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="8" dataCellStyle="Hiperlink"/>
+    <tableColumn id="3" xr3:uid="{62104941-F9E6-4824-97B5-2A48ACFEB884}" name="DATA ADMISSÃO" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{7271809A-319F-42CA-B3C0-541D631C23AA}" name="CARGO" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{0D375E2B-128D-4616-9AC4-B297337904BE}" name="GÊNERO" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{D8BE0E60-84AD-463D-A75B-55784F722626}" name="DATA DE NASCIMENTO" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{E5B3B1C5-E3FE-4003-AFCB-892540E2CB2D}" name="ATIVO" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A2F90783-8FA5-44E6-902F-D2631455F863}" name="Tabela16" displayName="Tabela16" ref="A1:H10" totalsRowShown="0" headerRowDxfId="40" dataDxfId="38" headerRowBorderDxfId="39" tableBorderDxfId="37" totalsRowBorderDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A2F90783-8FA5-44E6-902F-D2631455F863}" name="Tabela16" displayName="Tabela16" ref="A1:H10" totalsRowShown="0" headerRowDxfId="54" dataDxfId="52" headerRowBorderDxfId="53" tableBorderDxfId="51" totalsRowBorderDxfId="50">
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{768F854A-5408-4125-ABB5-04309C1E992F}" name="NOME COLABORADOR" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{5703C70A-67A0-420C-8C56-BC1592D6E703}" name="LOGIN COBMAIS" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{DF42236E-E428-4E7E-8C0F-8FB649F7174E}" name="ID SRS" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{EDB7C7D2-DF21-4268-935C-54378627C765}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="32" dataCellStyle="Hiperlink"/>
-    <tableColumn id="5" xr3:uid="{BC348017-3650-438A-BEFC-0AD6B25F7913}" name="DATA ADMISSÃO" dataDxfId="31"/>
-    <tableColumn id="6" xr3:uid="{79099123-196D-4D7F-BC12-1750373F8BE7}" name="CARGO" dataDxfId="30"/>
-    <tableColumn id="7" xr3:uid="{B8BF3F1E-3900-40B8-A0DD-66AF054BA62E}" name="GÊNERO" dataDxfId="29"/>
-    <tableColumn id="8" xr3:uid="{CD375B43-FAD7-4BDD-883B-3832718D88AE}" name="DATA DE NASCIMENTO" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{768F854A-5408-4125-ABB5-04309C1E992F}" name="NOME COLABORADOR" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{5703C70A-67A0-420C-8C56-BC1592D6E703}" name="LOGIN COBMAIS" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{DF42236E-E428-4E7E-8C0F-8FB649F7174E}" name="ID SRS" dataDxfId="47"/>
+    <tableColumn id="4" xr3:uid="{EDB7C7D2-DF21-4268-935C-54378627C765}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="46" dataCellStyle="Hiperlink"/>
+    <tableColumn id="5" xr3:uid="{BC348017-3650-438A-BEFC-0AD6B25F7913}" name="DATA ADMISSÃO" dataDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{79099123-196D-4D7F-BC12-1750373F8BE7}" name="CARGO" dataDxfId="44"/>
+    <tableColumn id="7" xr3:uid="{B8BF3F1E-3900-40B8-A0DD-66AF054BA62E}" name="GÊNERO" dataDxfId="43"/>
+    <tableColumn id="8" xr3:uid="{CD375B43-FAD7-4BDD-883B-3832718D88AE}" name="DATA DE NASCIMENTO" dataDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FBB1541A-6781-4544-BAB0-5A041D74860B}" name="Tabela1" displayName="Tabela1" ref="A1:H11" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24" totalsRowBorderDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FBB1541A-6781-4544-BAB0-5A041D74860B}" name="Tabela1" displayName="Tabela1" ref="A1:H11" totalsRowShown="0" headerRowDxfId="41" dataDxfId="39" headerRowBorderDxfId="40" tableBorderDxfId="38" totalsRowBorderDxfId="37">
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{60D0EC89-8A2E-490A-978A-989A9A1AFAC4}" name="NOME COLABORADOR" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{FBA2D0CD-99DF-427D-AE03-B74EAB39AA22}" name="LOGIN COBMAIS" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{F2CF9483-22C3-42E8-B5AB-EEC3774BE064}" name="ID SRS" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{EE579FB2-AB21-4497-B64C-E2167B0962F3}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="19" dataCellStyle="Hiperlink"/>
-    <tableColumn id="5" xr3:uid="{B6867804-B6AE-46EB-A574-B4331B3696C6}" name="DATA ADMISSÃO" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{2FB9A362-9746-46F7-BDDD-BA66E147AA63}" name="CARGO" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{AB53F85B-1857-4632-96CF-D7FF26BBB5E1}" name="GÊNERO" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{BCD78FD1-77BC-4ABA-BE2C-E1CD7CB6FA90}" name="DATA DE NASCIMENTO" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{60D0EC89-8A2E-490A-978A-989A9A1AFAC4}" name="NOME COLABORADOR" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{FBA2D0CD-99DF-427D-AE03-B74EAB39AA22}" name="LOGIN COBMAIS" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{F2CF9483-22C3-42E8-B5AB-EEC3774BE064}" name="ID SRS" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{EE579FB2-AB21-4497-B64C-E2167B0962F3}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="33" dataCellStyle="Hiperlink"/>
+    <tableColumn id="5" xr3:uid="{B6867804-B6AE-46EB-A574-B4331B3696C6}" name="DATA ADMISSÃO" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{2FB9A362-9746-46F7-BDDD-BA66E147AA63}" name="CARGO" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{AB53F85B-1857-4632-96CF-D7FF26BBB5E1}" name="GÊNERO" dataDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{BCD78FD1-77BC-4ABA-BE2C-E1CD7CB6FA90}" name="DATA DE NASCIMENTO" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1D55DD1B-9805-445D-B0FB-49EB5B17158F}" name="Tabela4" displayName="Tabela4" ref="A1:H8" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1D55DD1B-9805-445D-B0FB-49EB5B17158F}" name="Tabela4" displayName="Tabela4" ref="A1:H8" totalsRowShown="0" headerRowDxfId="28" dataDxfId="26" headerRowBorderDxfId="27" tableBorderDxfId="25">
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{98D2A8DD-E7E8-4CA5-9D7C-A68BCB105DD5}" name="NOME COLABORADOR" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{0DDDD88C-0256-4ADC-835D-BAF9E1771F41}" name="LOGIN COBMAIS" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{667A536D-2400-480A-9A3B-63CE8EAD5006}" name="ID SRS" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{2A867807-C22A-4295-9585-6E0FE2595863}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="7" dataCellStyle="Hiperlink"/>
-    <tableColumn id="5" xr3:uid="{99FE0ACB-7445-412D-9881-14D47142D1EB}" name="DATA ADMISSÃO" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{A1972CB8-1C10-421C-B582-B987EDCF66BA}" name="CARGO" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{482E0C1A-6FB1-4C8C-9C2F-2CB668047032}" name="GÊNERO" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{C0D136A6-27BF-407A-A6D7-F302EF0B6D23}" name="DATA DE NASCIMENTO" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{98D2A8DD-E7E8-4CA5-9D7C-A68BCB105DD5}" name="NOME COLABORADOR" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{0DDDD88C-0256-4ADC-835D-BAF9E1771F41}" name="LOGIN COBMAIS" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{667A536D-2400-480A-9A3B-63CE8EAD5006}" name="ID SRS" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{2A867807-C22A-4295-9585-6E0FE2595863}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="21" dataCellStyle="Hiperlink"/>
+    <tableColumn id="5" xr3:uid="{99FE0ACB-7445-412D-9881-14D47142D1EB}" name="DATA ADMISSÃO" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{A1972CB8-1C10-421C-B582-B987EDCF66BA}" name="CARGO" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{482E0C1A-6FB1-4C8C-9C2F-2CB668047032}" name="GÊNERO" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{C0D136A6-27BF-407A-A6D7-F302EF0B6D23}" name="DATA DE NASCIMENTO" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2048,7 +2114,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47.28515625" style="2" bestFit="1" customWidth="1"/>
@@ -2060,7 +2126,7 @@
     <col min="8" max="8" width="28.85546875" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -2085,8 +2151,11 @@
       <c r="H1" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="14" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
         <v>118</v>
       </c>
@@ -2111,8 +2180,11 @@
       <c r="H2" s="7">
         <v>36973</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2" s="30" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>104</v>
       </c>
@@ -2137,8 +2209,11 @@
       <c r="H3" s="7">
         <v>36723</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3" s="30" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
         <v>94</v>
       </c>
@@ -2163,8 +2238,11 @@
       <c r="H4" s="7">
         <v>40913</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I4" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>117</v>
       </c>
@@ -2189,8 +2267,11 @@
       <c r="H5" s="7">
         <v>33299</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I5" s="30" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
         <v>101</v>
       </c>
@@ -2215,8 +2296,11 @@
       <c r="H6" s="7">
         <v>37002</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I6" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>105</v>
       </c>
@@ -2241,8 +2325,11 @@
       <c r="H7" s="7">
         <v>33623</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I7" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
         <v>106</v>
       </c>
@@ -2267,8 +2354,11 @@
       <c r="H8" s="7">
         <v>37301</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I8" s="30" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>107</v>
       </c>
@@ -2293,8 +2383,11 @@
       <c r="H9" s="7">
         <v>34244</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I9" s="30" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
         <v>108</v>
       </c>
@@ -2319,8 +2412,11 @@
       <c r="H10" s="7">
         <v>34880</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I10" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>109</v>
       </c>
@@ -2345,8 +2441,11 @@
       <c r="H11" s="7">
         <v>36697</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I11" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
         <v>110</v>
       </c>
@@ -2371,8 +2470,11 @@
       <c r="H12" s="7">
         <v>24073</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I12" s="30" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>111</v>
       </c>
@@ -2397,8 +2499,11 @@
       <c r="H13" s="7">
         <v>33190</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I13" s="30" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
         <v>148</v>
       </c>
@@ -2419,8 +2524,11 @@
         <v>74</v>
       </c>
       <c r="H14" s="7"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I14" s="30" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>112</v>
       </c>
@@ -2445,8 +2553,11 @@
       <c r="H15" s="7">
         <v>36276</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I15" s="30" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="25" t="s">
         <v>113</v>
       </c>
@@ -2471,8 +2582,11 @@
       <c r="H16" s="7">
         <v>35467</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I16" s="30" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>126</v>
       </c>
@@ -2497,8 +2611,11 @@
       <c r="H17" s="7">
         <v>38287</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I17" s="30" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
         <v>114</v>
       </c>
@@ -2521,8 +2638,11 @@
         <v>74</v>
       </c>
       <c r="H18" s="7"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I18" s="32" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>130</v>
       </c>
@@ -2541,8 +2661,11 @@
         <v>75</v>
       </c>
       <c r="H19" s="7"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I19" s="32" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="25" t="s">
         <v>135</v>
       </c>
@@ -2561,8 +2684,11 @@
         <v>75</v>
       </c>
       <c r="H20" s="7"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I20" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>131</v>
       </c>
@@ -2583,8 +2709,11 @@
         <v>74</v>
       </c>
       <c r="H21" s="7"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I21" s="32" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="25" t="s">
         <v>129</v>
       </c>
@@ -2605,8 +2734,11 @@
         <v>74</v>
       </c>
       <c r="H22" s="7"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I22" s="32" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>140</v>
       </c>
@@ -2627,8 +2759,11 @@
         <v>75</v>
       </c>
       <c r="H23" s="7"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I23" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="25" t="s">
         <v>142</v>
       </c>
@@ -2649,8 +2784,11 @@
         <v>75</v>
       </c>
       <c r="H24" s="7"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I24" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>144</v>
       </c>
@@ -2671,8 +2809,11 @@
         <v>74</v>
       </c>
       <c r="H25" s="7"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I25" s="32" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
         <v>146</v>
       </c>
@@ -2693,8 +2834,11 @@
         <v>74</v>
       </c>
       <c r="H26" s="7"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I26" s="32" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>141</v>
       </c>
@@ -2719,8 +2863,11 @@
       <c r="H27" s="7">
         <v>37360</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I27" s="32" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="25" t="s">
         <v>157</v>
       </c>
@@ -2743,8 +2890,11 @@
         <v>74</v>
       </c>
       <c r="H28" s="7"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I28" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>158</v>
       </c>
@@ -2767,8 +2917,11 @@
         <v>74</v>
       </c>
       <c r="H29" s="7"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I29" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>159</v>
       </c>
@@ -2789,8 +2942,11 @@
         <v>74</v>
       </c>
       <c r="H30" s="7"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I30" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>165</v>
       </c>
@@ -2811,8 +2967,11 @@
         <v>75</v>
       </c>
       <c r="H31" s="7"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I31" s="31" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>156</v>
       </c>
@@ -2833,6 +2992,9 @@
         <v>75</v>
       </c>
       <c r="H32" s="7"/>
+      <c r="I32" s="31" t="s">
+        <v>181</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -3135,13 +3297,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4">
-    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{C85BE59B-44B0-48AC-A486-5203C818149A}"/>

</xml_diff>

<commit_message>
Atualiza colaboradores e quartis de metas
</commit_message>
<xml_diff>
--- a/Base de colaboradores.xlsx
+++ b/Base de colaboradores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samuel.victor\Desktop\ANALISE DO HISTORICO DE OPERADORES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A76E6B45-DF0F-468A-A355-49A330A08F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3FA8677-3AB3-4A19-81F7-415EABD88D70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-3270" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="JUDICIAL" sheetId="1" r:id="rId1"/>
@@ -886,6 +886,634 @@
   <dxfs count="55">
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <fill>
         <patternFill patternType="none">
           <bgColor auto="1"/>
@@ -928,36 +1556,6 @@
           <color indexed="64"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
@@ -1127,13 +1725,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -1157,600 +1748,9 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FF000000"/>
+        <bottom style="thin">
+          <color indexed="64"/>
         </bottom>
       </border>
     </dxf>
@@ -1781,68 +1781,68 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E73478C6-AA34-456B-BB72-ADF60DB89795}" name="Tabela2" displayName="Tabela2" ref="A1:I17" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" headerRowBorderDxfId="13" tableBorderDxfId="14" totalsRowBorderDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E73478C6-AA34-456B-BB72-ADF60DB89795}" name="Tabela2" displayName="Tabela2" ref="A1:I17" totalsRowShown="0" headerRowDxfId="54" dataDxfId="52" headerRowBorderDxfId="53" tableBorderDxfId="51" totalsRowBorderDxfId="50">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H16">
     <sortCondition ref="A15:A16"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{44B01074-0E94-49D7-A638-9DE941BE9A75}" name="NOME COLABORADOR" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{F9A57807-E92F-4AC4-A57B-5E3A31CA8C2B}" name="LOGIN COBMAIS" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{3D537BF0-580E-42DC-AAC3-452BD19ECF16}" name="ID SRS" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{AE32C28F-E44F-4C85-B0D8-0877E06AAD05}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="8" dataCellStyle="Hiperlink"/>
-    <tableColumn id="3" xr3:uid="{62104941-F9E6-4824-97B5-2A48ACFEB884}" name="DATA ADMISSÃO" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{7271809A-319F-42CA-B3C0-541D631C23AA}" name="CARGO" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{0D375E2B-128D-4616-9AC4-B297337904BE}" name="GÊNERO" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{D8BE0E60-84AD-463D-A75B-55784F722626}" name="DATA DE NASCIMENTO" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{E5B3B1C5-E3FE-4003-AFCB-892540E2CB2D}" name="ATIVO" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{44B01074-0E94-49D7-A638-9DE941BE9A75}" name="NOME COLABORADOR" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{F9A57807-E92F-4AC4-A57B-5E3A31CA8C2B}" name="LOGIN COBMAIS" dataDxfId="48"/>
+    <tableColumn id="2" xr3:uid="{3D537BF0-580E-42DC-AAC3-452BD19ECF16}" name="ID SRS" dataDxfId="47"/>
+    <tableColumn id="6" xr3:uid="{AE32C28F-E44F-4C85-B0D8-0877E06AAD05}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="46" dataCellStyle="Hiperlink"/>
+    <tableColumn id="3" xr3:uid="{62104941-F9E6-4824-97B5-2A48ACFEB884}" name="DATA ADMISSÃO" dataDxfId="45"/>
+    <tableColumn id="8" xr3:uid="{7271809A-319F-42CA-B3C0-541D631C23AA}" name="CARGO" dataDxfId="44"/>
+    <tableColumn id="7" xr3:uid="{0D375E2B-128D-4616-9AC4-B297337904BE}" name="GÊNERO" dataDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{D8BE0E60-84AD-463D-A75B-55784F722626}" name="DATA DE NASCIMENTO" dataDxfId="42"/>
+    <tableColumn id="9" xr3:uid="{E5B3B1C5-E3FE-4003-AFCB-892540E2CB2D}" name="ATIVO" dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A2F90783-8FA5-44E6-902F-D2631455F863}" name="Tabela16" displayName="Tabela16" ref="A1:H10" totalsRowShown="0" headerRowDxfId="54" dataDxfId="52" headerRowBorderDxfId="53" tableBorderDxfId="51" totalsRowBorderDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A2F90783-8FA5-44E6-902F-D2631455F863}" name="Tabela16" displayName="Tabela16" ref="A1:H10" totalsRowShown="0" headerRowDxfId="37" dataDxfId="35" headerRowBorderDxfId="36" tableBorderDxfId="34" totalsRowBorderDxfId="33">
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{768F854A-5408-4125-ABB5-04309C1E992F}" name="NOME COLABORADOR" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{5703C70A-67A0-420C-8C56-BC1592D6E703}" name="LOGIN COBMAIS" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{DF42236E-E428-4E7E-8C0F-8FB649F7174E}" name="ID SRS" dataDxfId="47"/>
-    <tableColumn id="4" xr3:uid="{EDB7C7D2-DF21-4268-935C-54378627C765}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="46" dataCellStyle="Hiperlink"/>
-    <tableColumn id="5" xr3:uid="{BC348017-3650-438A-BEFC-0AD6B25F7913}" name="DATA ADMISSÃO" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{79099123-196D-4D7F-BC12-1750373F8BE7}" name="CARGO" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{B8BF3F1E-3900-40B8-A0DD-66AF054BA62E}" name="GÊNERO" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{CD375B43-FAD7-4BDD-883B-3832718D88AE}" name="DATA DE NASCIMENTO" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{768F854A-5408-4125-ABB5-04309C1E992F}" name="NOME COLABORADOR" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{5703C70A-67A0-420C-8C56-BC1592D6E703}" name="LOGIN COBMAIS" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{DF42236E-E428-4E7E-8C0F-8FB649F7174E}" name="ID SRS" dataDxfId="30"/>
+    <tableColumn id="4" xr3:uid="{EDB7C7D2-DF21-4268-935C-54378627C765}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="29" dataCellStyle="Hiperlink"/>
+    <tableColumn id="5" xr3:uid="{BC348017-3650-438A-BEFC-0AD6B25F7913}" name="DATA ADMISSÃO" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{79099123-196D-4D7F-BC12-1750373F8BE7}" name="CARGO" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{B8BF3F1E-3900-40B8-A0DD-66AF054BA62E}" name="GÊNERO" dataDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{CD375B43-FAD7-4BDD-883B-3832718D88AE}" name="DATA DE NASCIMENTO" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FBB1541A-6781-4544-BAB0-5A041D74860B}" name="Tabela1" displayName="Tabela1" ref="A1:H11" totalsRowShown="0" headerRowDxfId="41" dataDxfId="39" headerRowBorderDxfId="40" tableBorderDxfId="38" totalsRowBorderDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FBB1541A-6781-4544-BAB0-5A041D74860B}" name="Tabela1" displayName="Tabela1" ref="A1:H11" totalsRowShown="0" headerRowDxfId="24" dataDxfId="22" headerRowBorderDxfId="23" tableBorderDxfId="21" totalsRowBorderDxfId="20">
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{60D0EC89-8A2E-490A-978A-989A9A1AFAC4}" name="NOME COLABORADOR" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{FBA2D0CD-99DF-427D-AE03-B74EAB39AA22}" name="LOGIN COBMAIS" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{F2CF9483-22C3-42E8-B5AB-EEC3774BE064}" name="ID SRS" dataDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{EE579FB2-AB21-4497-B64C-E2167B0962F3}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="33" dataCellStyle="Hiperlink"/>
-    <tableColumn id="5" xr3:uid="{B6867804-B6AE-46EB-A574-B4331B3696C6}" name="DATA ADMISSÃO" dataDxfId="32"/>
-    <tableColumn id="6" xr3:uid="{2FB9A362-9746-46F7-BDDD-BA66E147AA63}" name="CARGO" dataDxfId="31"/>
-    <tableColumn id="7" xr3:uid="{AB53F85B-1857-4632-96CF-D7FF26BBB5E1}" name="GÊNERO" dataDxfId="30"/>
-    <tableColumn id="8" xr3:uid="{BCD78FD1-77BC-4ABA-BE2C-E1CD7CB6FA90}" name="DATA DE NASCIMENTO" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{60D0EC89-8A2E-490A-978A-989A9A1AFAC4}" name="NOME COLABORADOR" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{FBA2D0CD-99DF-427D-AE03-B74EAB39AA22}" name="LOGIN COBMAIS" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{F2CF9483-22C3-42E8-B5AB-EEC3774BE064}" name="ID SRS" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{EE579FB2-AB21-4497-B64C-E2167B0962F3}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="16" dataCellStyle="Hiperlink"/>
+    <tableColumn id="5" xr3:uid="{B6867804-B6AE-46EB-A574-B4331B3696C6}" name="DATA ADMISSÃO" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{2FB9A362-9746-46F7-BDDD-BA66E147AA63}" name="CARGO" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{AB53F85B-1857-4632-96CF-D7FF26BBB5E1}" name="GÊNERO" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{BCD78FD1-77BC-4ABA-BE2C-E1CD7CB6FA90}" name="DATA DE NASCIMENTO" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1D55DD1B-9805-445D-B0FB-49EB5B17158F}" name="Tabela4" displayName="Tabela4" ref="A1:H8" totalsRowShown="0" headerRowDxfId="28" dataDxfId="26" headerRowBorderDxfId="27" tableBorderDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1D55DD1B-9805-445D-B0FB-49EB5B17158F}" name="Tabela4" displayName="Tabela4" ref="A1:H8" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8">
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{98D2A8DD-E7E8-4CA5-9D7C-A68BCB105DD5}" name="NOME COLABORADOR" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{0DDDD88C-0256-4ADC-835D-BAF9E1771F41}" name="LOGIN COBMAIS" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{667A536D-2400-480A-9A3B-63CE8EAD5006}" name="ID SRS" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{2A867807-C22A-4295-9585-6E0FE2595863}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="21" dataCellStyle="Hiperlink"/>
-    <tableColumn id="5" xr3:uid="{99FE0ACB-7445-412D-9881-14D47142D1EB}" name="DATA ADMISSÃO" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{A1972CB8-1C10-421C-B582-B987EDCF66BA}" name="CARGO" dataDxfId="19"/>
-    <tableColumn id="7" xr3:uid="{482E0C1A-6FB1-4C8C-9C2F-2CB668047032}" name="GÊNERO" dataDxfId="18"/>
-    <tableColumn id="8" xr3:uid="{C0D136A6-27BF-407A-A6D7-F302EF0B6D23}" name="DATA DE NASCIMENTO" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{98D2A8DD-E7E8-4CA5-9D7C-A68BCB105DD5}" name="NOME COLABORADOR" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{0DDDD88C-0256-4ADC-835D-BAF9E1771F41}" name="LOGIN COBMAIS" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{667A536D-2400-480A-9A3B-63CE8EAD5006}" name="ID SRS" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{2A867807-C22A-4295-9585-6E0FE2595863}" name="E-MAIL VINCULADO AO LOGIN DO SRS" dataDxfId="4" dataCellStyle="Hiperlink"/>
+    <tableColumn id="5" xr3:uid="{99FE0ACB-7445-412D-9881-14D47142D1EB}" name="DATA ADMISSÃO" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{A1972CB8-1C10-421C-B582-B987EDCF66BA}" name="CARGO" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{482E0C1A-6FB1-4C8C-9C2F-2CB668047032}" name="GÊNERO" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{C0D136A6-27BF-407A-A6D7-F302EF0B6D23}" name="DATA DE NASCIMENTO" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2943,7 +2943,7 @@
       </c>
       <c r="H30" s="7"/>
       <c r="I30" s="31" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -3297,13 +3297,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="3"/>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{C85BE59B-44B0-48AC-A486-5203C818149A}"/>

</xml_diff>